<commit_message>
chore: regenerate RegBriefings test data from full 50-test combined run
All 6 RegBriefings sub-modules run together cleanly via the dedicated
entry point: python run_tests.py --feature regbriefings -> 50/50
passing against RC, confirming no cross-sub-feature interference.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_data/RegBriefings/RegBriefings My Briefs/RegBriefings My Briefs_Test_Cases.xlsx
+++ b/test_data/RegBriefings/RegBriefings My Briefs/RegBriefings My Briefs_Test_Cases.xlsx
@@ -787,7 +787,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>My Briefs correctly shows 2 'Full Story in Regfollower' link(s).</t>
+          <t>My Briefs correctly shows 66 'Full Story in Regfollower' link(s).</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -1020,7 +1020,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Clicking 'World Tax Brief' navigated to https://regplus.kaz.com.bd/regbrief/home/wtaBriefings.</t>
+          <t>Clicking 'World Tax Brief' navigated to https://regplusrc.reganalytics.com/regbrief/home/wtaBriefings.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -1079,7 +1079,7 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Clicking 'Transfer Pricing Brief' navigated to https://regplus.kaz.com.bd/regbrief/home/tpaBriefings.</t>
+          <t>Clicking 'Transfer Pricing Brief' navigated to https://regplusrc.reganalytics.com/regbrief/home/tpaBriefings.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
@@ -1138,7 +1138,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Clicking 'Tax Treaty Brief' navigated to https://regplus.kaz.com.bd/regbrief/home/taxTreaties.</t>
+          <t>Clicking 'Tax Treaty Brief' navigated to https://regplusrc.reganalytics.com/regbrief/home/taxTreaties.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1197,7 +1197,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Clicking 'Archive' navigated to https://regplus.kaz.com.bd/regbrief/pastBriefingYearly.</t>
+          <t>Clicking 'Archive' navigated to https://regplusrc.reganalytics.com/regbrief/pastBriefingYearly.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">

</xml_diff>